<commit_message>
Videre med SVM note og forløb.
</commit_message>
<xml_diff>
--- a/undervisningsforlob/virker_medicinen/svm_excel_opgave8.xlsx
+++ b/undervisningsforlob/virker_medicinen/svm_excel_opgave8.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Bruger\Documents\GitHub\aalborg-intelligence.github.io\undervisningsforlob\virker_medicinen\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B16E1671-7932-4132-A716-03C35CAFDC6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9FFAAD0D-7E05-4031-910C-9EE9287ACB72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14720" yWindow="1530" windowWidth="16720" windowHeight="9970" xr2:uid="{954B3886-323B-4922-A0CE-9BF915E070C4}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{954B3886-323B-4922-A0CE-9BF915E070C4}"/>
   </bookViews>
   <sheets>
     <sheet name="Ark1" sheetId="1" r:id="rId1"/>
@@ -256,7 +256,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
@@ -269,9 +269,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -645,17 +642,17 @@
       </c>
       <c r="E5">
         <f>D5*($H$5*B5+$H$6*C5+$H$7)</f>
-        <v>2.2360706305904281</v>
+        <v>0.7</v>
       </c>
       <c r="G5" s="4" t="s">
         <v>5</v>
       </c>
       <c r="H5" s="6">
-        <v>-0.44721567517772598</v>
+        <v>1</v>
       </c>
       <c r="J5">
         <f>H5*SQRT(5)</f>
-        <v>-1.0000046503008606</v>
+        <v>2.2360679774997898</v>
       </c>
     </row>
     <row r="6" spans="2:10" x14ac:dyDescent="0.35">
@@ -670,17 +667,17 @@
       </c>
       <c r="E6">
         <f t="shared" ref="E6:E13" si="0">D6*($H$5*B6+$H$6*C6+$H$7)</f>
-        <v>-2.5938389058885067</v>
+        <v>-0.7</v>
       </c>
       <c r="G6" s="7" t="s">
         <v>6</v>
       </c>
       <c r="H6" s="8">
-        <v>-0.89442601930032395</v>
+        <v>1</v>
       </c>
       <c r="J6">
         <f>H6*SQRT(5)</f>
-        <v>-1.9999973800000634</v>
+        <v>2.2360679774997898</v>
       </c>
     </row>
     <row r="7" spans="2:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -695,17 +692,17 @@
       </c>
       <c r="E7">
         <f t="shared" si="0"/>
-        <v>-1.6994155521157466</v>
+        <v>-1.2</v>
       </c>
       <c r="G7" s="9" t="s">
         <v>7</v>
       </c>
       <c r="H7" s="11">
-        <v>2.2360690312738898</v>
+        <v>1</v>
       </c>
       <c r="J7">
         <f>H7*SQRT(5)</f>
-        <v>5.0000023563105209</v>
+        <v>2.2360679774997898</v>
       </c>
     </row>
     <row r="8" spans="2:10" x14ac:dyDescent="0.35">
@@ -720,7 +717,7 @@
       </c>
       <c r="E8">
         <f t="shared" si="0"/>
-        <v>-2.5043973701694999</v>
+        <v>-0.6</v>
       </c>
     </row>
     <row r="9" spans="2:10" x14ac:dyDescent="0.35">
@@ -735,7 +732,7 @@
       </c>
       <c r="E9">
         <f t="shared" si="0"/>
-        <v>1.1627556756914499</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="10" spans="2:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -750,29 +747,29 @@
       </c>
       <c r="E10">
         <f t="shared" si="0"/>
-        <v>0.49193589466345067</v>
+        <v>3.4</v>
       </c>
     </row>
     <row r="11" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B11" s="12">
+      <c r="B11" s="7">
         <v>1.5</v>
       </c>
-      <c r="C11" s="13">
+      <c r="C11">
         <v>0.7</v>
       </c>
-      <c r="D11" s="14">
+      <c r="D11" s="8">
         <v>1</v>
       </c>
       <c r="E11">
         <f t="shared" si="0"/>
-        <v>0.939147304997074</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="12" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B12" s="12">
+      <c r="B12" s="7">
         <v>1.4</v>
       </c>
-      <c r="C12" s="13">
+      <c r="C12">
         <v>1.2</v>
       </c>
       <c r="D12">
@@ -780,18 +777,18 @@
       </c>
       <c r="E12">
         <f t="shared" si="0"/>
-        <v>-0.5366558628646847</v>
+        <v>-3.5999999999999996</v>
       </c>
       <c r="G12">
         <f>H5^2+H6^2</f>
-        <v>0.99999976412609271</v>
+        <v>2</v>
       </c>
     </row>
     <row r="13" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B13" s="12">
+      <c r="B13" s="7">
         <v>0.2</v>
       </c>
-      <c r="C13" s="13">
+      <c r="C13">
         <v>0.2</v>
       </c>
       <c r="D13">
@@ -799,7 +796,7 @@
       </c>
       <c r="E13">
         <f t="shared" si="0"/>
-        <v>-1.9677406923782799</v>
+        <v>-1.4</v>
       </c>
     </row>
     <row r="17" spans="4:5" x14ac:dyDescent="0.35">
@@ -808,7 +805,7 @@
       </c>
       <c r="E17">
         <f>MIN(E5:E13)</f>
-        <v>-2.5938389058885067</v>
+        <v>-3.5999999999999996</v>
       </c>
     </row>
   </sheetData>

</xml_diff>